<commit_message>
update Test case Excel file
</commit_message>
<xml_diff>
--- a/TestData/OrangeHRM_Automation_Test_Cases.xlsx
+++ b/TestData/OrangeHRM_Automation_Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IC_Projects\Excersise\OrangeHRMHybridAutomationFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACBDBE59-E65F-4476-A55B-BDAB356EE8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C892F6A5-D2E9-4EF3-8F86-468D07D369C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,9 +78,6 @@
 3.Click Login</t>
   </si>
   <si>
-    <t>Username='', Password=''</t>
-  </si>
-  <si>
     <t>'Required' validation displayed</t>
   </si>
   <si>
@@ -110,9 +107,6 @@
 3.Click Login</t>
   </si>
   <si>
-    <t>Admin,''</t>
-  </si>
-  <si>
     <t>LG003</t>
   </si>
   <si>
@@ -228,6 +222,12 @@
   </si>
   <si>
     <t>Pass</t>
+  </si>
+  <si>
+    <t>Username=, Password=</t>
+  </si>
+  <si>
+    <t>Admin,</t>
   </si>
 </sst>
 </file>
@@ -624,7 +624,7 @@
         <v>11</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -647,271 +647,271 @@
         <v>17</v>
       </c>
       <c r="G2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
       <c r="N2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
         <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>26</v>
       </c>
       <c r="E3" t="s">
         <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
         <v>19</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>20</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>21</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>22</v>
       </c>
-      <c r="L3" t="s">
-        <v>23</v>
-      </c>
       <c r="N3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" t="s">
         <v>30</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>31</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>32</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>33</v>
       </c>
-      <c r="G4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" t="s">
-        <v>35</v>
-      </c>
       <c r="I4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" t="s">
         <v>20</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>21</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>22</v>
       </c>
-      <c r="L4" t="s">
-        <v>23</v>
-      </c>
       <c r="N4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
       </c>
       <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
         <v>37</v>
       </c>
-      <c r="D5" t="s">
+      <c r="G5" t="s">
         <v>38</v>
       </c>
-      <c r="E5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" t="s">
-        <v>39</v>
-      </c>
-      <c r="G5" t="s">
-        <v>40</v>
-      </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" t="s">
         <v>20</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>21</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>22</v>
       </c>
-      <c r="L5" t="s">
-        <v>23</v>
-      </c>
       <c r="N5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
       </c>
       <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
         <v>42</v>
       </c>
-      <c r="D6" t="s">
+      <c r="G6" t="s">
         <v>43</v>
       </c>
-      <c r="E6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>45</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>46</v>
       </c>
-      <c r="I6" t="s">
-        <v>47</v>
-      </c>
-      <c r="J6" t="s">
-        <v>48</v>
-      </c>
       <c r="K6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6" t="s">
         <v>22</v>
       </c>
-      <c r="L6" t="s">
-        <v>23</v>
-      </c>
       <c r="N6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
       </c>
       <c r="C7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
         <v>50</v>
       </c>
-      <c r="D7" t="s">
+      <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="E7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>52</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>53</v>
       </c>
-      <c r="H7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" t="s">
-        <v>55</v>
-      </c>
       <c r="J7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7" t="s">
         <v>22</v>
       </c>
-      <c r="L7" t="s">
-        <v>23</v>
-      </c>
       <c r="N7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
         <v>56</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>58</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
         <v>59</v>
       </c>
-      <c r="E8" t="s">
+      <c r="G8" t="s">
         <v>60</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>61</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" t="s">
         <v>62</v>
       </c>
-      <c r="H8" t="s">
+      <c r="K8" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8" t="s">
         <v>63</v>
       </c>
-      <c r="I8" t="s">
-        <v>47</v>
-      </c>
-      <c r="J8" t="s">
-        <v>64</v>
-      </c>
-      <c r="K8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" t="s">
+      <c r="N8" t="s">
         <v>65</v>
-      </c>
-      <c r="N8" t="s">
-        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>